<commit_message>
Fix GitHub Pages load: relative assets, static data map, clean JSON
Map deck fetches to data/*.json; ship map CSS/JS under assets/;
sanitize live-feed; war-day snapshots; exports relative. No demo.
</commit_message>
<xml_diff>
--- a/export/big-grin-swallows.xlsx
+++ b/export/big-grin-swallows.xlsx
@@ -35,7 +35,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-13T21:34Z</t>
+          <t>2026-07-13T21:53Z</t>
         </is>
       </c>
     </row>
@@ -95,7 +95,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LETHAL KILL/REKILL. Cook Field FAT. Queue reburn. Burn. Scrub. Destroy to wall outlet. Terror does not exist. God Bless.</t>
+          <t>WAR DAY · REAL hunt · LETHAL KILL/REKILL · no demo · no fake · God Bless.</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1432</t>
+          <t>3773</t>
         </is>
       </c>
     </row>
@@ -25079,12 +25079,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>462</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-13T21:34Z</t>
+          <t>2026-07-13T21:53Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
Escalate: all 265 kill dossiers DEAD DEAD + rekill +3/cycle
Wartime C++ rewrite: status DEAD, dead:true, every_kill_rekill,
rekill_count climbs for piss. kill-escalate board. No soft EATEN.
</commit_message>
<xml_diff>
--- a/export/big-grin-swallows.xlsx
+++ b/export/big-grin-swallows.xlsx
@@ -35,7 +35,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-13T21:53Z</t>
+          <t>2026-07-13T22:28Z</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3773</t>
+          <t>12118</t>
         </is>
       </c>
     </row>
@@ -15442,7 +15442,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>ironclad_mesh_fail \u00b7 hostess7_not_meshed \u00b7 liar_risk \u00b7 destroy_all</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · ironclad_mesh_fail \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 hostess7_not_meshed \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 liar_risk \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 destroy_all</t>
         </is>
       </c>
     </row>
@@ -15459,7 +15459,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>OUSTED</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -15499,7 +15499,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>terrorist_hacker_kit \u00b7 permanent_oust</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · terrorist_hacker_kit \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 permanent_oust</t>
         </is>
       </c>
     </row>
@@ -15556,7 +15556,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -15613,7 +15613,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -15670,7 +15670,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -15727,7 +15727,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -15784,7 +15784,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -15841,7 +15841,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -15898,7 +15898,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -15955,7 +15955,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16012,7 +16012,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16069,7 +16069,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16126,7 +16126,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16183,7 +16183,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16240,7 +16240,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16297,7 +16297,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16354,7 +16354,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16411,7 +16411,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16468,7 +16468,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16525,7 +16525,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16582,7 +16582,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16639,7 +16639,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16696,7 +16696,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -16753,7 +16753,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16810,7 +16810,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16867,7 +16867,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16924,7 +16924,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>rf_unhealthy_forever</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rf_unhealthy_forever</t>
         </is>
       </c>
     </row>
@@ -16981,7 +16981,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Active</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Active</t>
         </is>
       </c>
     </row>
@@ -17038,7 +17038,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>rekill_all_registered:High</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:High</t>
         </is>
       </c>
     </row>
@@ -17095,7 +17095,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Fresh</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Fresh</t>
         </is>
       </c>
     </row>
@@ -17152,7 +17152,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Fresh</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Fresh</t>
         </is>
       </c>
     </row>
@@ -17209,7 +17209,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Fresh</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Fresh</t>
         </is>
       </c>
     </row>
@@ -17266,7 +17266,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Censys</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Censys</t>
         </is>
       </c>
     </row>
@@ -17323,7 +17323,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>rekill_same_host_validated</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_same_host_validated</t>
         </is>
       </c>
     </row>
@@ -17380,7 +17380,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>wartime_rekill</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · wartime_rekill</t>
         </is>
       </c>
     </row>
@@ -17437,7 +17437,7 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Active</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Active</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17494,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>rekill_all_registered:Fresh</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · rekill_all_registered:Fresh</t>
         </is>
       </c>
     </row>
@@ -17511,7 +17511,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -17551,7 +17551,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Parent-child process policy + untrusted path scoring \u2014 not signature AV</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Parent-child process policy + untrusted path scoring \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 not signature AV</t>
         </is>
       </c>
     </row>
@@ -17568,7 +17568,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -17608,7 +17608,7 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>KILL \u00b7 crush autoscan source</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · KILL \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 crush autoscan source</t>
         </is>
       </c>
     </row>
@@ -17625,7 +17625,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -17665,7 +17665,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>KILL \u00b7 sever machine-precision C2</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · KILL \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 sever machine-precision C2</t>
         </is>
       </c>
     </row>
@@ -17682,7 +17682,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -17722,7 +17722,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Sever wire \u00b7 restore DNS/DHCP truth</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Sever wire \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 restore DNS/DHCP truth</t>
         </is>
       </c>
     </row>
@@ -17739,7 +17739,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -17779,7 +17779,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>KILL \u00b7 stop shaped exfil</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · KILL \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 stop shaped exfil</t>
         </is>
       </c>
     </row>
@@ -17796,7 +17796,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -17836,7 +17836,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>KILL \u00b7 eradicate temp-binary chain</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · KILL \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 eradicate temp-binary chain</t>
         </is>
       </c>
     </row>
@@ -17848,12 +17848,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Stacked weak signals \u2014 ML-managed C2</t>
+          <t>Stacked weak signals \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 ML-managed C2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -17893,7 +17893,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>KILL \u00b7 destroy stacked C2</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · KILL \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 destroy stacked C2</t>
         </is>
       </c>
     </row>
@@ -17910,7 +17910,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -17950,7 +17950,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Beacon pattern axis \u22657 + timing entropy collapse on flow key</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Beacon pattern axis \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u22657 + timing entropy collapse on flow key</t>
         </is>
       </c>
     </row>
@@ -17967,7 +17967,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -18007,7 +18007,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Honeypot paths + exploit-port DPI + listener surge correlation</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Honeypot paths + exploit-port DPI + listener surge correlation</t>
         </is>
       </c>
     </row>
@@ -18024,7 +18024,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Gateway integrity + DNS query entropy + resolv.conf truth cycle</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Gateway integrity + DNS query entropy + resolv.conf truth cycle</t>
         </is>
       </c>
     </row>
@@ -18081,7 +18081,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -18121,7 +18121,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18138,7 +18138,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -18178,7 +18178,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18195,7 +18195,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -18235,7 +18235,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18252,7 +18252,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -18292,7 +18292,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18309,7 +18309,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -18349,7 +18349,7 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18366,7 +18366,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18423,7 +18423,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -18463,7 +18463,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18480,7 +18480,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -18520,7 +18520,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18537,7 +18537,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -18577,7 +18577,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18594,7 +18594,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -18634,7 +18634,7 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18651,7 +18651,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -18691,7 +18691,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18708,7 +18708,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -18748,7 +18748,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18765,7 +18765,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -18805,7 +18805,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18822,7 +18822,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -18862,7 +18862,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18879,7 +18879,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -18919,7 +18919,7 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18936,7 +18936,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -18976,7 +18976,7 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -18993,7 +18993,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -19033,7 +19033,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19050,7 +19050,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -19090,7 +19090,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19107,7 +19107,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -19147,7 +19147,7 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19164,7 +19164,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -19204,7 +19204,7 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19221,7 +19221,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -19261,7 +19261,7 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19278,7 +19278,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -19318,7 +19318,7 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19335,7 +19335,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -19375,7 +19375,7 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19392,7 +19392,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -19432,7 +19432,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19449,7 +19449,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -19489,7 +19489,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19506,7 +19506,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -19546,7 +19546,7 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19563,7 +19563,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -19603,7 +19603,7 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19620,7 +19620,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -19660,7 +19660,7 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19677,7 +19677,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -19717,7 +19717,7 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19734,7 +19734,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -19774,7 +19774,7 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19791,7 +19791,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -19831,7 +19831,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19848,7 +19848,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -19888,7 +19888,7 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19905,7 +19905,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -19945,7 +19945,7 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -19962,7 +19962,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -20002,7 +20002,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20019,7 +20019,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -20059,7 +20059,7 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20076,7 +20076,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -20116,7 +20116,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20133,7 +20133,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -20173,7 +20173,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20190,7 +20190,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -20230,7 +20230,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20247,7 +20247,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -20287,7 +20287,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20304,7 +20304,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -20344,7 +20344,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20361,7 +20361,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -20401,7 +20401,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20418,7 +20418,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20475,7 +20475,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -20515,7 +20515,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20532,7 +20532,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -20572,7 +20572,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20589,7 +20589,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -20629,7 +20629,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20646,7 +20646,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -20686,7 +20686,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20703,7 +20703,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -20743,7 +20743,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20760,7 +20760,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -20800,7 +20800,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20817,7 +20817,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -20857,7 +20857,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20874,7 +20874,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20931,7 +20931,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -20971,7 +20971,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -20988,7 +20988,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -21028,7 +21028,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21045,7 +21045,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -21085,7 +21085,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21102,7 +21102,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -21142,7 +21142,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21159,7 +21159,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -21199,7 +21199,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21216,7 +21216,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -21256,7 +21256,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21273,7 +21273,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -21313,7 +21313,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21330,7 +21330,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -21370,7 +21370,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21387,7 +21387,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -21427,7 +21427,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21444,7 +21444,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -21484,7 +21484,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21501,7 +21501,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -21541,7 +21541,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21558,7 +21558,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -21598,7 +21598,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21615,7 +21615,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -21655,7 +21655,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21672,7 +21672,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -21712,7 +21712,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21729,7 +21729,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -21769,7 +21769,7 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21786,7 +21786,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -21826,7 +21826,7 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21843,7 +21843,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -21883,7 +21883,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21900,7 +21900,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -21940,7 +21940,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -21957,7 +21957,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -21997,7 +21997,7 @@
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22014,7 +22014,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -22054,7 +22054,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22071,7 +22071,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -22111,7 +22111,7 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22128,7 +22128,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22185,7 +22185,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -22225,7 +22225,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22242,7 +22242,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -22282,7 +22282,7 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22299,7 +22299,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -22339,7 +22339,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22356,7 +22356,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -22396,7 +22396,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22413,7 +22413,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -22453,7 +22453,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22470,7 +22470,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -22510,7 +22510,7 @@
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22527,7 +22527,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -22567,7 +22567,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22584,7 +22584,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -22624,7 +22624,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22641,7 +22641,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -22681,7 +22681,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -22738,7 +22738,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22755,7 +22755,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -22795,7 +22795,7 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22812,7 +22812,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -22852,7 +22852,7 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22869,7 +22869,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -22909,7 +22909,7 @@
       </c>
       <c r="K133" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22926,7 +22926,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -22966,7 +22966,7 @@
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -22983,7 +22983,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -23023,7 +23023,7 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23040,7 +23040,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -23080,7 +23080,7 @@
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23097,7 +23097,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -23137,7 +23137,7 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23154,7 +23154,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -23194,7 +23194,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23211,7 +23211,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -23251,7 +23251,7 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23268,7 +23268,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -23308,7 +23308,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23325,7 +23325,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -23365,7 +23365,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23382,7 +23382,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -23422,7 +23422,7 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23439,7 +23439,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -23479,7 +23479,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23496,7 +23496,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -23536,7 +23536,7 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -23593,7 +23593,7 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23610,7 +23610,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -23650,7 +23650,7 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23667,7 +23667,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -23707,7 +23707,7 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23724,7 +23724,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -23764,7 +23764,7 @@
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23781,7 +23781,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -23821,7 +23821,7 @@
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23838,7 +23838,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -23878,7 +23878,7 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -23895,7 +23895,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -23935,7 +23935,7 @@
       </c>
       <c r="K151" t="inlineStr">
         <is>
-          <t>Per-host egress baseline + gatekeeper bandwidth/stream axes</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Per-host egress baseline + gatekeeper bandwidth/stream axes</t>
         </is>
       </c>
     </row>
@@ -23952,7 +23952,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -23992,24 +23992,24 @@
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>threat-stacked weak signals \u2014 ml-managed c2</t>
+          <t>threat-stacked weak signals \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 ml-managed c2</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Stacked weak signals \u2014 ML-managed C2</t>
+          <t>Stacked weak signals \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 ML-managed C2</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -24049,7 +24049,7 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Correlation score + multi-vector same peer \u2014 meta but actionable</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Correlation score + multi-vector same peer \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 meta but actionable</t>
         </is>
       </c>
     </row>
@@ -24066,7 +24066,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -24123,7 +24123,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -24163,7 +24163,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -24180,7 +24180,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -24220,7 +24220,7 @@
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -24237,7 +24237,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -24277,7 +24277,7 @@
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -24294,7 +24294,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -24334,7 +24334,7 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>permanent_list</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · permanent_list</t>
         </is>
       </c>
     </row>
@@ -24351,7 +24351,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -24391,7 +24391,7 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Honorability + browser awareness + auth velocity \u2014 not content ML alone</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Honorability + browser awareness + auth velocity \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 not content ML alone</t>
         </is>
       </c>
     </row>
@@ -24408,7 +24408,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -24448,7 +24448,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Sever wire \u00b7 block fraud egress</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Sever wire \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u00b7 block fraud egress</t>
         </is>
       </c>
     </row>
@@ -24465,7 +24465,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -24505,7 +24505,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
@@ -24522,7 +24522,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -24562,7 +24562,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
@@ -24579,7 +24579,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -24619,7 +24619,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
@@ -24636,7 +24636,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -24676,7 +24676,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
@@ -24693,7 +24693,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -24733,24 +24733,24 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>threat-collision guard \u2014 7 foreign hooks, 0 eradicated on sight</t>
+          <t>threat-collision guard \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 7 foreign hooks, 0 eradicated on sight</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Collision guard \u2014 7 foreign hooks, 0 eradicated on sight</t>
+          <t>Collision guard \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 7 foreign hooks, 0 eradicated on sight</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -24790,7 +24790,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>ISP CPE resolvers, foreign DHCP OFFERs, and rogue listeners that try to hijack planetary DNS/DHCP authority get permanent blocks, nft drops, and SIGKILL. No qua</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · ISP CPE resolvers, foreign DHCP OFFERs, and rogue listeners that try to hijack planetary DNS/DHCP authority get permanent blocks, nft drops, and SIGKILL. No qua</t>
         </is>
       </c>
     </row>
@@ -24807,7 +24807,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -24847,7 +24847,7 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
@@ -24864,7 +24864,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -24904,7 +24904,7 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · Orphan panel JSON subprocesses and duplicate publish queues burn CPU when C2 is down. Purge kills them; Big Grin Pwnership records why. Never remove from kill l</t>
         </is>
       </c>
     </row>
@@ -24921,7 +24921,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -24961,7 +24961,7 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>dump_bash_state piles, GROK_AGENT shells, sleep infinity, subagent storms, and panel subprocess duplicates get SIGKILL. GrokSpawnKiller never sleeps \u2014 every kil</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · dump_bash_state piles, GROK_AGENT shells, sleep infinity, subagent storms, and panel subprocess duplicates get SIGKILL. GrokSpawnKiller never sleeps \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 every kil</t>
         </is>
       </c>
     </row>
@@ -24978,7 +24978,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>EATEN</t>
+          <t>DEAD</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -25018,7 +25018,7 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>dump_bash_state piles, GROK_AGENT shells, sleep infinity, subagent storms, and panel subprocess duplicates get SIGKILL. GrokSpawnKiller never sleeps \u2014 every kil</t>
+          <t>ESCALATE_REKILL · DEAD_DEAD · rekill+3 · cycle 1 · dump_bash_state piles, GROK_AGENT shells, sleep infinity, subagent storms, and panel subprocess duplicates get SIGKILL. GrokSpawnKiller never sleeps \\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\\u2014 every kil</t>
         </is>
       </c>
     </row>
@@ -25079,12 +25079,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>1235</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-13T21:53Z</t>
+          <t>2026-07-13T22:28Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
Live 265 DEAD dossiers · clean export-only controls
Refresh kill-dossiers from C++ wartime, prefer live pack in deck,
export bar is CSV/JSON/Excel/ODS only, 4s poll for live counts.
</commit_message>
<xml_diff>
--- a/export/big-grin-swallows.xlsx
+++ b/export/big-grin-swallows.xlsx
@@ -35,7 +35,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-13T22:28Z</t>
+          <t>2026-07-14T00:16Z</t>
         </is>
       </c>
     </row>
@@ -95,7 +95,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>WAR DAY · REAL hunt · LETHAL KILL/REKILL · no demo · no fake · God Bless.</t>
+          <t>COOKED · Field UDP fries global servers to WALL OUTLET · nothing left · no storage · no room · HATED · PISSED · God Bless</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>12118</t>
+          <t>89572</t>
         </is>
       </c>
     </row>
@@ -25079,12 +25079,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1235</t>
+          <t>7193</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-13T22:28Z</t>
+          <t>2026-07-14T00:16Z</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>